<commit_message>
Small UserStories formatting changes
Fitted text by changing width of cell & Wrapping
Added bold to top two
</commit_message>
<xml_diff>
--- a/userStoriesUpdated.xlsx
+++ b/userStoriesUpdated.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luke\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Downloads\GitRepositories\Software-Engineering-Project-G1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A665767-FC93-4EAA-835D-16BCEF463D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F3B784-45FC-4628-86CF-F7FE45037F05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -634,19 +634,40 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -982,1892 +1003,2011 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDD9AED8-E474-4BF9-9553-A6EDBA2E72AE}">
-  <dimension ref="A1:I176"/>
+  <dimension ref="A1:J176"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
-    <col min="2" max="2" width="61.28515625" customWidth="1"/>
-    <col min="3" max="3" width="49.28515625" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="80.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="217.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="B2" s="6"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B4" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C6" t="s">
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B6" s="7"/>
+      <c r="C6" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C7" t="s">
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B7" s="7"/>
+      <c r="C7" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B8" s="7"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
         <v>2</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C12" t="s">
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="7"/>
+      <c r="C12" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C13" t="s">
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="7"/>
+      <c r="C13" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15">
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="6"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
         <v>3</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B16" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19">
+      <c r="A19" s="2">
         <v>4</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="A23" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24">
+      <c r="A24" s="2">
         <v>1</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28">
+      <c r="A28" s="2">
         <v>2</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B29" s="4" t="s">
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+    </row>
+    <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B29" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B31" s="4"/>
-      <c r="C31" s="4" t="s">
+      <c r="B31" s="7"/>
+      <c r="C31" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33">
+      <c r="A33" s="2">
         <v>3</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37">
+      <c r="A37" s="2">
         <v>4</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
-      <c r="I38" s="4"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B40" s="4"/>
-      <c r="C40" s="4" t="s">
+      <c r="B40" s="7"/>
+      <c r="C40" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
-      <c r="I40" s="4"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="4"/>
-      <c r="C41" s="4" t="s">
+      <c r="B41" s="7"/>
+      <c r="C41" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B42" s="4"/>
-      <c r="C42" s="4" t="s">
+      <c r="B42" s="7"/>
+      <c r="C42" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
-      <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
-      <c r="I42" s="4"/>
+      <c r="D42" s="1"/>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B43" s="4"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="4"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="1"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+      <c r="I43" s="1"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
+      <c r="A44" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-      <c r="I44" s="4"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="1"/>
+      <c r="D44" s="1"/>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+      <c r="I44" s="1"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45">
+      <c r="A45" s="2">
         <v>1</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
+      <c r="D45" s="1"/>
+      <c r="E45" s="1"/>
+      <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+      <c r="I45" s="1"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-      <c r="I46" s="4"/>
+      <c r="D46" s="1"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="I46" s="1"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C47" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+      <c r="I47" s="1"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B48" s="4"/>
-      <c r="C48" s="5" t="s">
+      <c r="B48" s="7"/>
+      <c r="C48" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4"/>
+      <c r="D48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="I48" s="1"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B49" s="4"/>
-      <c r="C49" s="5" t="s">
+      <c r="B49" s="7"/>
+      <c r="C49" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
-      <c r="I49" s="4"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+      <c r="I49" s="1"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B50" s="4"/>
-      <c r="C50" s="5" t="s">
+      <c r="B50" s="7"/>
+      <c r="C50" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D50" s="4"/>
-      <c r="E50" s="4"/>
-      <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
+      <c r="D50" s="1"/>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B51" s="4"/>
-      <c r="C51" s="5" t="s">
+      <c r="B51" s="7"/>
+      <c r="C51" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
+      <c r="D51" s="1"/>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+      <c r="I51" s="1"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52">
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="2">
         <v>2</v>
       </c>
-      <c r="B52" s="4"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
-      <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
-      <c r="I52" s="4"/>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B53" s="5" t="s">
+      <c r="B53" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C53" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
-      <c r="I53" s="4"/>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+      <c r="I53" s="1"/>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B54" s="5" t="s">
+      <c r="B54" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
-      <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
-      <c r="I54" s="4"/>
+      <c r="D54" s="1"/>
+      <c r="E54" s="1"/>
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+      <c r="I54" s="1"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
-      <c r="I55" s="4"/>
+      <c r="D55" s="1"/>
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+      <c r="I55" s="1"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B56" s="4"/>
-      <c r="C56" s="5" t="s">
+      <c r="B56" s="7"/>
+      <c r="C56" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
-      <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
-      <c r="I56" s="4"/>
+      <c r="D56" s="1"/>
+      <c r="E56" s="1"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+      <c r="I56" s="1"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B57" s="4"/>
-      <c r="C57" s="5" t="s">
+      <c r="B57" s="7"/>
+      <c r="C57" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4"/>
-      <c r="I57" s="4"/>
+      <c r="D57" s="1"/>
+      <c r="E57" s="1"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
+      <c r="I57" s="1"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B58" s="4"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
+      <c r="B58" s="7"/>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59">
+      <c r="A59" s="2">
         <v>3</v>
       </c>
-      <c r="B59" s="5" t="s">
+      <c r="B59" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="C59" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
-      <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
-      <c r="I59" s="4"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1"/>
+      <c r="I59" s="1"/>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="C60" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
-      <c r="I60" s="4"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+      <c r="I60" s="1"/>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B61" s="5" t="s">
+      <c r="B61" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="C61" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
-      <c r="F61" s="4"/>
-      <c r="G61" s="4"/>
-      <c r="H61" s="4"/>
-      <c r="I61" s="4"/>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
+      <c r="H61" s="1"/>
+      <c r="I61" s="1"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B62" s="4"/>
-      <c r="C62" s="5" t="s">
+      <c r="B62" s="7"/>
+      <c r="C62" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
-      <c r="F62" s="4"/>
-      <c r="G62" s="4"/>
-      <c r="H62" s="4"/>
-      <c r="I62" s="4"/>
+      <c r="D62" s="1"/>
+      <c r="E62" s="1"/>
+      <c r="F62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="H62" s="1"/>
+      <c r="I62" s="1"/>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B63" s="4"/>
-      <c r="C63" s="5" t="s">
+      <c r="B63" s="7"/>
+      <c r="C63" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-      <c r="I63" s="4"/>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1"/>
+      <c r="I63" s="1"/>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B64" s="4"/>
-      <c r="C64" s="5" t="s">
+      <c r="B64" s="7"/>
+      <c r="C64" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D64" s="4"/>
-      <c r="E64" s="4"/>
-      <c r="F64" s="4"/>
-      <c r="G64" s="4"/>
-      <c r="H64" s="4"/>
-      <c r="I64" s="4"/>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1"/>
+      <c r="F64" s="1"/>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1"/>
+      <c r="I64" s="1"/>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B65" s="4"/>
-      <c r="C65" s="5" t="s">
+      <c r="B65" s="7"/>
+      <c r="C65" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D65" s="4"/>
-      <c r="E65" s="4"/>
-      <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
-      <c r="H65" s="4"/>
-      <c r="I65" s="4"/>
+      <c r="D65" s="1"/>
+      <c r="E65" s="1"/>
+      <c r="F65" s="1"/>
+      <c r="G65" s="1"/>
+      <c r="H65" s="1"/>
+      <c r="I65" s="1"/>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B66" s="4"/>
-      <c r="C66" s="4"/>
-      <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
-      <c r="F66" s="4"/>
-      <c r="G66" s="4"/>
-      <c r="H66" s="4"/>
-      <c r="I66" s="4"/>
+      <c r="B66" s="7"/>
+      <c r="C66" s="1"/>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1"/>
+      <c r="F66" s="1"/>
+      <c r="G66" s="1"/>
+      <c r="H66" s="1"/>
+      <c r="I66" s="1"/>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A67">
+      <c r="A67" s="2">
         <v>4</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C67" s="4" t="s">
+      <c r="C67" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D67" s="4"/>
-      <c r="E67" s="4"/>
-      <c r="F67" s="4"/>
-      <c r="G67" s="4"/>
-      <c r="H67" s="4"/>
-      <c r="I67" s="4"/>
+      <c r="D67" s="1"/>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1"/>
+      <c r="G67" s="1"/>
+      <c r="H67" s="1"/>
+      <c r="I67" s="1"/>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A68" s="3"/>
-      <c r="B68" s="5" t="s">
+      <c r="A68" s="10"/>
+      <c r="B68" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C68" s="4" t="s">
+      <c r="C68" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D68" s="4"/>
-      <c r="E68" s="4"/>
-      <c r="F68" s="4"/>
-      <c r="G68" s="4"/>
-      <c r="H68" s="4"/>
-      <c r="I68" s="4"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1"/>
+      <c r="F68" s="1"/>
+      <c r="G68" s="1"/>
+      <c r="H68" s="1"/>
+      <c r="I68" s="1"/>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A69" s="3"/>
-      <c r="B69" s="5" t="s">
+      <c r="A69" s="10"/>
+      <c r="B69" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C69" s="5" t="s">
+      <c r="C69" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D69" s="4"/>
-      <c r="E69" s="4"/>
-      <c r="F69" s="4"/>
-      <c r="G69" s="4"/>
-      <c r="H69" s="4"/>
-      <c r="I69" s="4"/>
+      <c r="D69" s="1"/>
+      <c r="E69" s="1"/>
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
+      <c r="I69" s="1"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B70" s="4"/>
-      <c r="C70" s="5" t="s">
+      <c r="B70" s="7"/>
+      <c r="C70" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D70" s="4"/>
-      <c r="E70" s="4"/>
-      <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-      <c r="I70" s="4"/>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
+      <c r="I70" s="1"/>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B71" s="4"/>
-      <c r="C71" s="5" t="s">
+      <c r="B71" s="7"/>
+      <c r="C71" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D71" s="4"/>
-      <c r="E71" s="4"/>
-      <c r="F71" s="4"/>
-      <c r="G71" s="4"/>
-      <c r="H71" s="4"/>
-      <c r="I71" s="4"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
+      <c r="F71" s="1"/>
+      <c r="G71" s="1"/>
+      <c r="H71" s="1"/>
+      <c r="I71" s="1"/>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B72" s="4"/>
-      <c r="C72" s="4"/>
-      <c r="D72" s="4"/>
-      <c r="E72" s="4"/>
-      <c r="F72" s="4"/>
-      <c r="G72" s="4"/>
-      <c r="H72" s="4"/>
-      <c r="I72" s="4"/>
+      <c r="B72" s="7"/>
+      <c r="C72" s="1"/>
+      <c r="D72" s="1"/>
+      <c r="E72" s="1"/>
+      <c r="F72" s="1"/>
+      <c r="G72" s="1"/>
+      <c r="H72" s="1"/>
+      <c r="I72" s="1"/>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+      <c r="A73" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B73" s="4"/>
-      <c r="C73" s="4"/>
-      <c r="D73" s="4"/>
-      <c r="E73" s="4"/>
-      <c r="F73" s="4"/>
-      <c r="G73" s="4"/>
-      <c r="H73" s="4"/>
-      <c r="I73" s="4"/>
+      <c r="B73" s="7"/>
+      <c r="C73" s="1"/>
+      <c r="D73" s="1"/>
+      <c r="E73" s="1"/>
+      <c r="F73" s="1"/>
+      <c r="G73" s="1"/>
+      <c r="H73" s="1"/>
+      <c r="I73" s="1"/>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A74">
+      <c r="A74" s="2">
         <v>1</v>
       </c>
-      <c r="B74" s="4" t="s">
+      <c r="B74" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C74" s="5" t="s">
+      <c r="C74" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D74" s="4"/>
-      <c r="E74" s="4"/>
-      <c r="F74" s="4"/>
-      <c r="G74" s="4"/>
-      <c r="H74" s="4"/>
-      <c r="I74" s="4"/>
+      <c r="D74" s="1"/>
+      <c r="E74" s="1"/>
+      <c r="F74" s="1"/>
+      <c r="G74" s="1"/>
+      <c r="H74" s="1"/>
+      <c r="I74" s="1"/>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B75" s="4" t="s">
+      <c r="B75" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C75" s="5" t="s">
+      <c r="C75" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D75" s="4"/>
-      <c r="E75" s="4"/>
-      <c r="F75" s="4"/>
-      <c r="G75" s="4"/>
-      <c r="H75" s="4"/>
-      <c r="I75" s="4"/>
+      <c r="D75" s="1"/>
+      <c r="E75" s="1"/>
+      <c r="F75" s="1"/>
+      <c r="G75" s="1"/>
+      <c r="H75" s="1"/>
+      <c r="I75" s="1"/>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B76" s="4" t="s">
+      <c r="B76" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C76" s="5" t="s">
+      <c r="C76" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D76" s="4"/>
-      <c r="E76" s="4"/>
-      <c r="F76" s="4"/>
-      <c r="G76" s="4"/>
-      <c r="H76" s="4"/>
-      <c r="I76" s="4"/>
+      <c r="D76" s="1"/>
+      <c r="E76" s="1"/>
+      <c r="F76" s="1"/>
+      <c r="G76" s="1"/>
+      <c r="H76" s="1"/>
+      <c r="I76" s="1"/>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B77" s="4"/>
-      <c r="C77" s="5" t="s">
+      <c r="B77" s="7"/>
+      <c r="C77" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D77" s="4"/>
-      <c r="E77" s="4"/>
-      <c r="F77" s="4"/>
-      <c r="G77" s="4"/>
-      <c r="H77" s="4"/>
-      <c r="I77" s="4"/>
+      <c r="D77" s="1"/>
+      <c r="E77" s="1"/>
+      <c r="F77" s="1"/>
+      <c r="G77" s="1"/>
+      <c r="H77" s="1"/>
+      <c r="I77" s="1"/>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B78" s="4"/>
-      <c r="C78" s="5" t="s">
+      <c r="B78" s="7"/>
+      <c r="C78" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D78" s="4"/>
-      <c r="E78" s="4"/>
-      <c r="F78" s="4"/>
-      <c r="G78" s="4"/>
-      <c r="H78" s="4"/>
-      <c r="I78" s="4"/>
+      <c r="D78" s="1"/>
+      <c r="E78" s="1"/>
+      <c r="F78" s="1"/>
+      <c r="G78" s="1"/>
+      <c r="H78" s="1"/>
+      <c r="I78" s="1"/>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B79" s="4"/>
-      <c r="C79" s="5" t="s">
+      <c r="B79" s="7"/>
+      <c r="C79" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D79" s="4"/>
-      <c r="E79" s="4"/>
-      <c r="F79" s="4"/>
-      <c r="G79" s="4"/>
-      <c r="H79" s="4"/>
-      <c r="I79" s="4"/>
+      <c r="D79" s="1"/>
+      <c r="E79" s="1"/>
+      <c r="F79" s="1"/>
+      <c r="G79" s="1"/>
+      <c r="H79" s="1"/>
+      <c r="I79" s="1"/>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B80" s="4"/>
-      <c r="C80" s="4"/>
-      <c r="D80" s="4"/>
-      <c r="E80" s="4"/>
-      <c r="F80" s="4"/>
-      <c r="G80" s="4"/>
-      <c r="H80" s="4"/>
-      <c r="I80" s="4"/>
+      <c r="B80" s="7"/>
+      <c r="C80" s="1"/>
+      <c r="D80" s="1"/>
+      <c r="E80" s="1"/>
+      <c r="F80" s="1"/>
+      <c r="G80" s="1"/>
+      <c r="H80" s="1"/>
+      <c r="I80" s="1"/>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A81">
+      <c r="A81" s="2">
         <v>2</v>
       </c>
-      <c r="B81" s="4" t="s">
+      <c r="B81" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C81" s="5" t="s">
+      <c r="C81" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D81" s="4"/>
-      <c r="E81" s="4"/>
-      <c r="F81" s="4"/>
-      <c r="G81" s="4"/>
-      <c r="H81" s="4"/>
-      <c r="I81" s="4"/>
+      <c r="D81" s="1"/>
+      <c r="E81" s="1"/>
+      <c r="F81" s="1"/>
+      <c r="G81" s="1"/>
+      <c r="H81" s="1"/>
+      <c r="I81" s="1"/>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B82" s="4" t="s">
+      <c r="B82" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="C82" s="5" t="s">
+      <c r="C82" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D82" s="4"/>
-      <c r="E82" s="4"/>
-      <c r="F82" s="4"/>
-      <c r="G82" s="4"/>
-      <c r="H82" s="4"/>
-      <c r="I82" s="4"/>
+      <c r="D82" s="1"/>
+      <c r="E82" s="1"/>
+      <c r="F82" s="1"/>
+      <c r="G82" s="1"/>
+      <c r="H82" s="1"/>
+      <c r="I82" s="1"/>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B83" s="4" t="s">
+      <c r="B83" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C83" s="5" t="s">
+      <c r="C83" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D83" s="4"/>
-      <c r="E83" s="4"/>
-      <c r="F83" s="4"/>
-      <c r="G83" s="4"/>
-      <c r="H83" s="4"/>
-      <c r="I83" s="4"/>
+      <c r="D83" s="1"/>
+      <c r="E83" s="1"/>
+      <c r="F83" s="1"/>
+      <c r="G83" s="1"/>
+      <c r="H83" s="1"/>
+      <c r="I83" s="1"/>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B84" s="4"/>
-      <c r="C84" s="5" t="s">
+      <c r="B84" s="7"/>
+      <c r="C84" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D84" s="4"/>
-      <c r="E84" s="4"/>
-      <c r="F84" s="4"/>
-      <c r="G84" s="4"/>
-      <c r="H84" s="4"/>
-      <c r="I84" s="4"/>
+      <c r="D84" s="1"/>
+      <c r="E84" s="1"/>
+      <c r="F84" s="1"/>
+      <c r="G84" s="1"/>
+      <c r="H84" s="1"/>
+      <c r="I84" s="1"/>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B85" s="4"/>
-      <c r="C85" s="5" t="s">
+      <c r="B85" s="7"/>
+      <c r="C85" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D85" s="4"/>
-      <c r="E85" s="4"/>
-      <c r="F85" s="4"/>
-      <c r="G85" s="4"/>
-      <c r="H85" s="4"/>
-      <c r="I85" s="4"/>
+      <c r="D85" s="1"/>
+      <c r="E85" s="1"/>
+      <c r="F85" s="1"/>
+      <c r="G85" s="1"/>
+      <c r="H85" s="1"/>
+      <c r="I85" s="1"/>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B86" s="4"/>
-      <c r="C86" s="4"/>
-      <c r="D86" s="4"/>
-      <c r="E86" s="4"/>
-      <c r="F86" s="4"/>
-      <c r="G86" s="4"/>
-      <c r="H86" s="4"/>
-      <c r="I86" s="4"/>
+      <c r="B86" s="7"/>
+      <c r="C86" s="1"/>
+      <c r="D86" s="1"/>
+      <c r="E86" s="1"/>
+      <c r="F86" s="1"/>
+      <c r="G86" s="1"/>
+      <c r="H86" s="1"/>
+      <c r="I86" s="1"/>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87">
+      <c r="A87" s="2">
         <v>3</v>
       </c>
-      <c r="B87" s="4" t="s">
+      <c r="B87" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C87" s="5" t="s">
+      <c r="C87" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D87" s="4"/>
-      <c r="E87" s="4"/>
-      <c r="F87" s="4"/>
-      <c r="G87" s="4"/>
-      <c r="H87" s="4"/>
-      <c r="I87" s="4"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="1"/>
+      <c r="F87" s="1"/>
+      <c r="G87" s="1"/>
+      <c r="H87" s="1"/>
+      <c r="I87" s="1"/>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B88" s="4" t="s">
+      <c r="B88" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C88" s="5" t="s">
+      <c r="C88" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D88" s="4"/>
-      <c r="E88" s="4"/>
-      <c r="F88" s="4"/>
-      <c r="G88" s="4"/>
-      <c r="H88" s="4"/>
-      <c r="I88" s="4"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="1"/>
+      <c r="F88" s="1"/>
+      <c r="G88" s="1"/>
+      <c r="H88" s="1"/>
+      <c r="I88" s="1"/>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B89" s="4" t="s">
+      <c r="B89" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C89" s="5" t="s">
+      <c r="C89" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D89" s="4"/>
-      <c r="E89" s="4"/>
-      <c r="F89" s="4"/>
-      <c r="G89" s="4"/>
-      <c r="H89" s="4"/>
-      <c r="I89" s="4"/>
+      <c r="D89" s="1"/>
+      <c r="E89" s="1"/>
+      <c r="F89" s="1"/>
+      <c r="G89" s="1"/>
+      <c r="H89" s="1"/>
+      <c r="I89" s="1"/>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B90" s="4"/>
-      <c r="C90" s="5" t="s">
+      <c r="B90" s="7"/>
+      <c r="C90" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D90" s="4"/>
-      <c r="E90" s="4"/>
-      <c r="F90" s="4"/>
-      <c r="G90" s="4"/>
-      <c r="H90" s="4"/>
-      <c r="I90" s="4"/>
+      <c r="D90" s="1"/>
+      <c r="E90" s="1"/>
+      <c r="F90" s="1"/>
+      <c r="G90" s="1"/>
+      <c r="H90" s="1"/>
+      <c r="I90" s="1"/>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B91" s="4"/>
-      <c r="C91" s="5" t="s">
+      <c r="B91" s="7"/>
+      <c r="C91" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D91" s="4"/>
-      <c r="E91" s="4"/>
-      <c r="F91" s="4"/>
-      <c r="G91" s="4"/>
-      <c r="H91" s="4"/>
-      <c r="I91" s="4"/>
+      <c r="D91" s="1"/>
+      <c r="E91" s="1"/>
+      <c r="F91" s="1"/>
+      <c r="G91" s="1"/>
+      <c r="H91" s="1"/>
+      <c r="I91" s="1"/>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B92" s="4"/>
-      <c r="C92" s="5" t="s">
+      <c r="B92" s="7"/>
+      <c r="C92" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D92" s="4"/>
-      <c r="E92" s="4"/>
-      <c r="F92" s="4"/>
-      <c r="G92" s="4"/>
-      <c r="H92" s="4"/>
-      <c r="I92" s="4"/>
+      <c r="D92" s="1"/>
+      <c r="E92" s="1"/>
+      <c r="F92" s="1"/>
+      <c r="G92" s="1"/>
+      <c r="H92" s="1"/>
+      <c r="I92" s="1"/>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B93" s="4"/>
-      <c r="C93" s="5" t="s">
+      <c r="B93" s="7"/>
+      <c r="C93" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D93" s="4"/>
-      <c r="E93" s="4"/>
-      <c r="F93" s="4"/>
-      <c r="G93" s="4"/>
-      <c r="H93" s="4"/>
-      <c r="I93" s="4"/>
+      <c r="D93" s="1"/>
+      <c r="E93" s="1"/>
+      <c r="F93" s="1"/>
+      <c r="G93" s="1"/>
+      <c r="H93" s="1"/>
+      <c r="I93" s="1"/>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B94" s="4"/>
-      <c r="C94" s="5" t="s">
+      <c r="B94" s="7"/>
+      <c r="C94" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D94" s="4"/>
-      <c r="E94" s="4"/>
-      <c r="F94" s="4"/>
-      <c r="G94" s="4"/>
-      <c r="H94" s="4"/>
-      <c r="I94" s="4"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="1"/>
+      <c r="F94" s="1"/>
+      <c r="G94" s="1"/>
+      <c r="H94" s="1"/>
+      <c r="I94" s="1"/>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B95" s="4"/>
-      <c r="C95" s="4"/>
-      <c r="D95" s="4"/>
-      <c r="E95" s="4"/>
-      <c r="F95" s="4"/>
-      <c r="G95" s="4"/>
-      <c r="H95" s="4"/>
-      <c r="I95" s="4"/>
+      <c r="B95" s="7"/>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="1"/>
+      <c r="F95" s="1"/>
+      <c r="G95" s="1"/>
+      <c r="H95" s="1"/>
+      <c r="I95" s="1"/>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A96">
+      <c r="A96" s="2">
         <v>4</v>
       </c>
-      <c r="B96" s="4" t="s">
+      <c r="B96" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C96" s="5" t="s">
+      <c r="C96" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="D96" s="4"/>
-      <c r="E96" s="4"/>
-      <c r="F96" s="4"/>
-      <c r="G96" s="4"/>
-      <c r="H96" s="4"/>
-      <c r="I96" s="4"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+      <c r="F96" s="1"/>
+      <c r="G96" s="1"/>
+      <c r="H96" s="1"/>
+      <c r="I96" s="1"/>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B97" s="4" t="s">
+      <c r="B97" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C97" s="5" t="s">
+      <c r="C97" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D97" s="4"/>
-      <c r="E97" s="4"/>
-      <c r="F97" s="4"/>
-      <c r="G97" s="4"/>
-      <c r="H97" s="4"/>
-      <c r="I97" s="4"/>
+      <c r="D97" s="1"/>
+      <c r="E97" s="1"/>
+      <c r="F97" s="1"/>
+      <c r="G97" s="1"/>
+      <c r="H97" s="1"/>
+      <c r="I97" s="1"/>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B98" s="4" t="s">
+      <c r="B98" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="C98" s="5" t="s">
+      <c r="C98" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D98" s="4"/>
-      <c r="E98" s="4"/>
-      <c r="F98" s="4"/>
-      <c r="G98" s="4"/>
-      <c r="H98" s="4"/>
-      <c r="I98" s="4"/>
+      <c r="D98" s="1"/>
+      <c r="E98" s="1"/>
+      <c r="F98" s="1"/>
+      <c r="G98" s="1"/>
+      <c r="H98" s="1"/>
+      <c r="I98" s="1"/>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B99" s="4"/>
-      <c r="C99" s="5" t="s">
+      <c r="B99" s="7"/>
+      <c r="C99" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="D99" s="4"/>
-      <c r="E99" s="4"/>
-      <c r="F99" s="4"/>
-      <c r="G99" s="4"/>
-      <c r="H99" s="4"/>
-      <c r="I99" s="4"/>
+      <c r="D99" s="1"/>
+      <c r="E99" s="1"/>
+      <c r="F99" s="1"/>
+      <c r="G99" s="1"/>
+      <c r="H99" s="1"/>
+      <c r="I99" s="1"/>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B100" s="4"/>
-      <c r="C100" s="4" t="s">
+      <c r="B100" s="7"/>
+      <c r="C100" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D100" s="4"/>
-      <c r="E100" s="4"/>
-      <c r="F100" s="4"/>
-      <c r="G100" s="4"/>
-      <c r="H100" s="4"/>
-      <c r="I100" s="4"/>
+      <c r="D100" s="1"/>
+      <c r="E100" s="1"/>
+      <c r="F100" s="1"/>
+      <c r="G100" s="1"/>
+      <c r="H100" s="1"/>
+      <c r="I100" s="1"/>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B101" s="4"/>
-      <c r="C101" s="4" t="s">
+      <c r="B101" s="7"/>
+      <c r="C101" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D101" s="4"/>
-      <c r="E101" s="4"/>
-      <c r="F101" s="4"/>
-      <c r="G101" s="4"/>
-      <c r="H101" s="4"/>
-      <c r="I101" s="4"/>
+      <c r="D101" s="1"/>
+      <c r="E101" s="1"/>
+      <c r="F101" s="1"/>
+      <c r="G101" s="1"/>
+      <c r="H101" s="1"/>
+      <c r="I101" s="1"/>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B102" s="4"/>
-      <c r="C102" s="5" t="s">
+      <c r="B102" s="7"/>
+      <c r="C102" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D102" s="4"/>
-      <c r="E102" s="4"/>
-      <c r="F102" s="4"/>
-      <c r="G102" s="4"/>
-      <c r="H102" s="4"/>
-      <c r="I102" s="4"/>
+      <c r="D102" s="1"/>
+      <c r="E102" s="1"/>
+      <c r="F102" s="1"/>
+      <c r="G102" s="1"/>
+      <c r="H102" s="1"/>
+      <c r="I102" s="1"/>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B103" s="4"/>
-      <c r="C103" s="5" t="s">
+      <c r="B103" s="7"/>
+      <c r="C103" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D103" s="4"/>
-      <c r="E103" s="4"/>
-      <c r="F103" s="4"/>
-      <c r="G103" s="4"/>
-      <c r="H103" s="4"/>
-      <c r="I103" s="4"/>
+      <c r="D103" s="1"/>
+      <c r="E103" s="1"/>
+      <c r="F103" s="1"/>
+      <c r="G103" s="1"/>
+      <c r="H103" s="1"/>
+      <c r="I103" s="1"/>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B104" s="4"/>
-      <c r="C104" s="4"/>
-      <c r="D104" s="4"/>
-      <c r="E104" s="4"/>
-      <c r="F104" s="4"/>
-      <c r="G104" s="4"/>
-      <c r="H104" s="4"/>
-      <c r="I104" s="4"/>
+      <c r="B104" s="7"/>
+      <c r="C104" s="1"/>
+      <c r="D104" s="1"/>
+      <c r="E104" s="1"/>
+      <c r="F104" s="1"/>
+      <c r="G104" s="1"/>
+      <c r="H104" s="1"/>
+      <c r="I104" s="1"/>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
+      <c r="A105" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B105" s="4"/>
-      <c r="C105" s="4"/>
-      <c r="D105" s="4"/>
-      <c r="E105" s="4"/>
-      <c r="F105" s="4"/>
-      <c r="G105" s="4"/>
-      <c r="H105" s="4"/>
-      <c r="I105" s="4"/>
+      <c r="B105" s="7"/>
+      <c r="C105" s="1"/>
+      <c r="D105" s="1"/>
+      <c r="E105" s="1"/>
+      <c r="F105" s="1"/>
+      <c r="G105" s="1"/>
+      <c r="H105" s="1"/>
+      <c r="I105" s="1"/>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A106">
+      <c r="A106" s="2">
         <v>1</v>
       </c>
-      <c r="B106" s="4" t="s">
+      <c r="B106" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C106" s="4" t="s">
+      <c r="C106" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="D106" s="4"/>
-      <c r="E106" s="4"/>
-      <c r="F106" s="4"/>
-      <c r="G106" s="4"/>
-      <c r="H106" s="4"/>
-      <c r="I106" s="4"/>
+      <c r="D106" s="1"/>
+      <c r="E106" s="1"/>
+      <c r="F106" s="1"/>
+      <c r="G106" s="1"/>
+      <c r="H106" s="1"/>
+      <c r="I106" s="1"/>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B107" s="4" t="s">
+      <c r="B107" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C107" s="4" t="s">
+      <c r="C107" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D107" s="4"/>
-      <c r="E107" s="4"/>
-      <c r="F107" s="4"/>
-      <c r="G107" s="4"/>
-      <c r="H107" s="4"/>
-      <c r="I107" s="4"/>
+      <c r="D107" s="1"/>
+      <c r="E107" s="1"/>
+      <c r="F107" s="1"/>
+      <c r="G107" s="1"/>
+      <c r="H107" s="1"/>
+      <c r="I107" s="1"/>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B108" s="4" t="s">
+      <c r="B108" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C108" s="4" t="s">
+      <c r="C108" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D108" s="4"/>
-      <c r="E108" s="4"/>
-      <c r="F108" s="4"/>
-      <c r="G108" s="4"/>
-      <c r="H108" s="4"/>
-      <c r="I108" s="4"/>
+      <c r="D108" s="1"/>
+      <c r="E108" s="1"/>
+      <c r="F108" s="1"/>
+      <c r="G108" s="1"/>
+      <c r="H108" s="1"/>
+      <c r="I108" s="1"/>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B109" s="4"/>
-      <c r="C109" s="4"/>
-      <c r="D109" s="4"/>
-      <c r="E109" s="4"/>
-      <c r="F109" s="4"/>
-      <c r="G109" s="4"/>
-      <c r="H109" s="4"/>
-      <c r="I109" s="4"/>
+      <c r="B109" s="7"/>
+      <c r="C109" s="1"/>
+      <c r="D109" s="1"/>
+      <c r="E109" s="1"/>
+      <c r="F109" s="1"/>
+      <c r="G109" s="1"/>
+      <c r="H109" s="1"/>
+      <c r="I109" s="1"/>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A110">
+      <c r="A110" s="2">
         <v>2</v>
       </c>
-      <c r="B110" s="4" t="s">
+      <c r="B110" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C110" s="4" t="s">
+      <c r="C110" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D110" s="4"/>
-      <c r="E110" s="4"/>
-      <c r="F110" s="4"/>
-      <c r="G110" s="4"/>
-      <c r="H110" s="4"/>
-      <c r="I110" s="4"/>
+      <c r="D110" s="1"/>
+      <c r="E110" s="1"/>
+      <c r="F110" s="1"/>
+      <c r="G110" s="1"/>
+      <c r="H110" s="1"/>
+      <c r="I110" s="1"/>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B111" s="4" t="s">
+      <c r="B111" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="C111" s="4" t="s">
+      <c r="C111" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D111" s="4"/>
-      <c r="E111" s="4"/>
-      <c r="F111" s="4"/>
-      <c r="G111" s="4"/>
-      <c r="H111" s="4"/>
-      <c r="I111" s="4"/>
+      <c r="D111" s="1"/>
+      <c r="E111" s="1"/>
+      <c r="F111" s="1"/>
+      <c r="G111" s="1"/>
+      <c r="H111" s="1"/>
+      <c r="I111" s="1"/>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B112" s="4" t="s">
+      <c r="B112" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="C112" s="4" t="s">
+      <c r="C112" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D112" s="4"/>
-      <c r="E112" s="4"/>
-      <c r="F112" s="4"/>
-      <c r="G112" s="4"/>
-      <c r="H112" s="4"/>
-      <c r="I112" s="4"/>
+      <c r="D112" s="1"/>
+      <c r="E112" s="1"/>
+      <c r="F112" s="1"/>
+      <c r="G112" s="1"/>
+      <c r="H112" s="1"/>
+      <c r="I112" s="1"/>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B113" s="4"/>
-      <c r="C113" s="4" t="s">
+      <c r="B113" s="7"/>
+      <c r="C113" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D113" s="4"/>
-      <c r="E113" s="4"/>
-      <c r="F113" s="4"/>
-      <c r="G113" s="4"/>
-      <c r="H113" s="4"/>
-      <c r="I113" s="4"/>
+      <c r="D113" s="1"/>
+      <c r="E113" s="1"/>
+      <c r="F113" s="1"/>
+      <c r="G113" s="1"/>
+      <c r="H113" s="1"/>
+      <c r="I113" s="1"/>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B114" s="4"/>
-      <c r="C114" s="4"/>
-      <c r="D114" s="4"/>
-      <c r="E114" s="4"/>
-      <c r="F114" s="4"/>
-      <c r="G114" s="4"/>
-      <c r="H114" s="4"/>
-      <c r="I114" s="4"/>
+      <c r="B114" s="7"/>
+      <c r="C114" s="1"/>
+      <c r="D114" s="1"/>
+      <c r="E114" s="1"/>
+      <c r="F114" s="1"/>
+      <c r="G114" s="1"/>
+      <c r="H114" s="1"/>
+      <c r="I114" s="1"/>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A115">
+      <c r="A115" s="2">
         <v>3</v>
       </c>
-      <c r="B115" s="4" t="s">
+      <c r="B115" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C115" s="4" t="s">
+      <c r="C115" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D115" s="4"/>
-      <c r="E115" s="4"/>
-      <c r="F115" s="4"/>
-      <c r="G115" s="4"/>
-      <c r="H115" s="4"/>
-      <c r="I115" s="4"/>
+      <c r="D115" s="1"/>
+      <c r="E115" s="1"/>
+      <c r="F115" s="1"/>
+      <c r="G115" s="1"/>
+      <c r="H115" s="1"/>
+      <c r="I115" s="1"/>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B116" s="4" t="s">
+      <c r="B116" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="C116" s="4" t="s">
+      <c r="C116" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D116" s="4"/>
-      <c r="E116" s="4"/>
-      <c r="F116" s="4"/>
-      <c r="G116" s="4"/>
-      <c r="H116" s="4"/>
-      <c r="I116" s="4"/>
+      <c r="D116" s="1"/>
+      <c r="E116" s="1"/>
+      <c r="F116" s="1"/>
+      <c r="G116" s="1"/>
+      <c r="H116" s="1"/>
+      <c r="I116" s="1"/>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B117" s="4" t="s">
+      <c r="B117" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="C117" s="4" t="s">
+      <c r="C117" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D117" s="4"/>
-      <c r="E117" s="4"/>
-      <c r="F117" s="4"/>
-      <c r="G117" s="4"/>
-      <c r="H117" s="4"/>
-      <c r="I117" s="4"/>
+      <c r="D117" s="1"/>
+      <c r="E117" s="1"/>
+      <c r="F117" s="1"/>
+      <c r="G117" s="1"/>
+      <c r="H117" s="1"/>
+      <c r="I117" s="1"/>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B118" s="4"/>
-      <c r="C118" s="4" t="s">
+      <c r="B118" s="7"/>
+      <c r="C118" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D118" s="4"/>
-      <c r="E118" s="4"/>
-      <c r="F118" s="4"/>
-      <c r="G118" s="4"/>
-      <c r="H118" s="4"/>
-      <c r="I118" s="4"/>
+      <c r="D118" s="1"/>
+      <c r="E118" s="1"/>
+      <c r="F118" s="1"/>
+      <c r="G118" s="1"/>
+      <c r="H118" s="1"/>
+      <c r="I118" s="1"/>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B119" s="4"/>
-      <c r="C119" s="4" t="s">
+      <c r="B119" s="7"/>
+      <c r="C119" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D119" s="4"/>
-      <c r="E119" s="4"/>
-      <c r="F119" s="4"/>
-      <c r="G119" s="4"/>
-      <c r="H119" s="4"/>
-      <c r="I119" s="4"/>
+      <c r="D119" s="1"/>
+      <c r="E119" s="1"/>
+      <c r="F119" s="1"/>
+      <c r="G119" s="1"/>
+      <c r="H119" s="1"/>
+      <c r="I119" s="1"/>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B120" s="4"/>
-      <c r="C120" s="4" t="s">
+      <c r="B120" s="7"/>
+      <c r="C120" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D120" s="4"/>
-      <c r="E120" s="4"/>
-      <c r="F120" s="4"/>
-      <c r="G120" s="4"/>
-      <c r="H120" s="4"/>
-      <c r="I120" s="4"/>
+      <c r="D120" s="1"/>
+      <c r="E120" s="1"/>
+      <c r="F120" s="1"/>
+      <c r="G120" s="1"/>
+      <c r="H120" s="1"/>
+      <c r="I120" s="1"/>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B121" s="4"/>
-      <c r="C121" s="4"/>
-      <c r="D121" s="4"/>
-      <c r="E121" s="4"/>
-      <c r="F121" s="4"/>
-      <c r="G121" s="4"/>
-      <c r="H121" s="4"/>
-      <c r="I121" s="4"/>
+      <c r="B121" s="7"/>
+      <c r="C121" s="1"/>
+      <c r="D121" s="1"/>
+      <c r="E121" s="1"/>
+      <c r="F121" s="1"/>
+      <c r="G121" s="1"/>
+      <c r="H121" s="1"/>
+      <c r="I121" s="1"/>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A122">
+      <c r="A122" s="2">
         <v>4</v>
       </c>
-      <c r="B122" s="4" t="s">
+      <c r="B122" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C122" s="4" t="s">
+      <c r="C122" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D122" s="4"/>
-      <c r="E122" s="4"/>
-      <c r="F122" s="4"/>
-      <c r="G122" s="4"/>
-      <c r="H122" s="4"/>
-      <c r="I122" s="4"/>
+      <c r="D122" s="1"/>
+      <c r="E122" s="1"/>
+      <c r="F122" s="1"/>
+      <c r="G122" s="1"/>
+      <c r="H122" s="1"/>
+      <c r="I122" s="1"/>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B123" s="4" t="s">
+      <c r="B123" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="C123" s="4" t="s">
+      <c r="C123" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D123" s="4"/>
-      <c r="E123" s="4"/>
-      <c r="F123" s="4"/>
-      <c r="G123" s="4"/>
-      <c r="H123" s="4"/>
-      <c r="I123" s="4"/>
+      <c r="D123" s="1"/>
+      <c r="E123" s="1"/>
+      <c r="F123" s="1"/>
+      <c r="G123" s="1"/>
+      <c r="H123" s="1"/>
+      <c r="I123" s="1"/>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B124" s="4" t="s">
+      <c r="B124" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="C124" s="4" t="s">
+      <c r="C124" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D124" s="4"/>
-      <c r="E124" s="4"/>
-      <c r="F124" s="4"/>
-      <c r="G124" s="4"/>
-      <c r="H124" s="4"/>
-      <c r="I124" s="4"/>
+      <c r="D124" s="1"/>
+      <c r="E124" s="1"/>
+      <c r="F124" s="1"/>
+      <c r="G124" s="1"/>
+      <c r="H124" s="1"/>
+      <c r="I124" s="1"/>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B125" s="4"/>
-      <c r="C125" s="4" t="s">
+      <c r="B125" s="7"/>
+      <c r="C125" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D125" s="4"/>
-      <c r="E125" s="4"/>
-      <c r="F125" s="4"/>
-      <c r="G125" s="4"/>
-      <c r="H125" s="4"/>
-      <c r="I125" s="4"/>
+      <c r="D125" s="1"/>
+      <c r="E125" s="1"/>
+      <c r="F125" s="1"/>
+      <c r="G125" s="1"/>
+      <c r="H125" s="1"/>
+      <c r="I125" s="1"/>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B126" s="4"/>
-      <c r="C126" s="4"/>
-      <c r="D126" s="4"/>
-      <c r="E126" s="4"/>
-      <c r="F126" s="4"/>
-      <c r="G126" s="4"/>
-      <c r="H126" s="4"/>
-      <c r="I126" s="4"/>
+      <c r="B126" s="7"/>
+      <c r="C126" s="1"/>
+      <c r="D126" s="1"/>
+      <c r="E126" s="1"/>
+      <c r="F126" s="1"/>
+      <c r="G126" s="1"/>
+      <c r="H126" s="1"/>
+      <c r="I126" s="1"/>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
+      <c r="A127" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B127" s="4"/>
-      <c r="C127" s="4"/>
-      <c r="D127" s="4"/>
-      <c r="E127" s="4"/>
-      <c r="F127" s="4"/>
-      <c r="G127" s="4"/>
-      <c r="H127" s="4"/>
-      <c r="I127" s="4"/>
+      <c r="B127" s="7"/>
+      <c r="C127" s="1"/>
+      <c r="D127" s="1"/>
+      <c r="E127" s="1"/>
+      <c r="F127" s="1"/>
+      <c r="G127" s="1"/>
+      <c r="H127" s="1"/>
+      <c r="I127" s="1"/>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A128">
+      <c r="A128" s="2">
         <v>1</v>
       </c>
-      <c r="B128" s="4" t="s">
+      <c r="B128" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C128" s="4" t="s">
+      <c r="C128" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D128" s="4"/>
-      <c r="E128" s="4"/>
-      <c r="F128" s="4"/>
-      <c r="G128" s="4"/>
-      <c r="H128" s="4"/>
-      <c r="I128" s="4"/>
+      <c r="D128" s="1"/>
+      <c r="E128" s="1"/>
+      <c r="F128" s="1"/>
+      <c r="G128" s="1"/>
+      <c r="H128" s="1"/>
+      <c r="I128" s="1"/>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B129" s="4" t="s">
+      <c r="B129" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C129" s="4"/>
-      <c r="D129" s="4"/>
-      <c r="E129" s="4"/>
-      <c r="F129" s="4"/>
-      <c r="G129" s="4"/>
-      <c r="H129" s="4"/>
-      <c r="I129" s="4"/>
+      <c r="C129" s="1"/>
+      <c r="D129" s="1"/>
+      <c r="E129" s="1"/>
+      <c r="F129" s="1"/>
+      <c r="G129" s="1"/>
+      <c r="H129" s="1"/>
+      <c r="I129" s="1"/>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B130" s="4" t="s">
+      <c r="B130" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="C130" s="4"/>
-      <c r="D130" s="4"/>
-      <c r="E130" s="4"/>
-      <c r="F130" s="4"/>
-      <c r="G130" s="4"/>
-      <c r="H130" s="4"/>
-      <c r="I130" s="4"/>
+      <c r="C130" s="1"/>
+      <c r="D130" s="1"/>
+      <c r="E130" s="1"/>
+      <c r="F130" s="1"/>
+      <c r="G130" s="1"/>
+      <c r="H130" s="1"/>
+      <c r="I130" s="1"/>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B131" s="6"/>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A132">
+      <c r="A132" s="2">
         <v>2</v>
       </c>
-      <c r="B132" s="5" t="s">
+      <c r="B132" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="C132" s="5" t="s">
+      <c r="C132" s="3" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B133" s="5" t="s">
+      <c r="B133" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="C133" s="5" t="s">
+      <c r="C133" s="3" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B134" s="5" t="s">
+      <c r="B134" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="C134" s="5" t="s">
+      <c r="C134" s="3" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C135" s="5" t="s">
+      <c r="B135" s="6"/>
+      <c r="C135" s="3" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C136" s="5" t="s">
+      <c r="B136" s="6"/>
+      <c r="C136" s="3" t="s">
         <v>142</v>
       </c>
     </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B137" s="6"/>
+    </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A138">
+      <c r="A138" s="2">
         <v>3</v>
       </c>
-      <c r="B138" s="5" t="s">
+      <c r="B138" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="C138" s="5" t="s">
+      <c r="C138" s="3" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B139" s="5" t="s">
+    <row r="139" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B139" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C139" s="5" t="s">
+      <c r="C139" s="3" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A140" s="6"/>
-      <c r="B140" s="5" t="s">
+      <c r="A140" s="11"/>
+      <c r="B140" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="C140" s="5"/>
+      <c r="C140" s="3"/>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B141" s="6"/>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
+      <c r="A142" s="2" t="s">
         <v>161</v>
       </c>
+      <c r="B142" s="6"/>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A143">
+      <c r="A143" s="2">
         <v>1</v>
       </c>
-      <c r="B143" s="5" t="s">
+      <c r="B143" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="C143" s="5" t="s">
+      <c r="C143" s="3" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B144" s="5" t="s">
+      <c r="B144" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="C144" s="5" t="s">
+      <c r="C144" s="3" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B145" s="5" t="s">
+      <c r="B145" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="C145" s="5"/>
+      <c r="C145" s="3"/>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B146" s="6"/>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A147">
+      <c r="A147" s="2">
         <v>2</v>
       </c>
-      <c r="B147" s="5" t="s">
+      <c r="B147" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="C147" s="5" t="s">
+      <c r="C147" s="3" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B148" s="5" t="s">
+      <c r="B148" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="C148" s="5" t="s">
+      <c r="C148" s="3" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B149" s="5" t="s">
+      <c r="B149" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C149" s="5" t="s">
+      <c r="C149" s="3" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C150" s="5" t="s">
+      <c r="B150" s="6"/>
+      <c r="C150" s="3" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C151" s="5" t="s">
+      <c r="B151" s="6"/>
+      <c r="C151" s="3" t="s">
         <v>160</v>
       </c>
     </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B152" s="6"/>
+    </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A153">
+      <c r="A153" s="2">
         <v>3</v>
       </c>
-      <c r="B153" s="5" t="s">
+      <c r="B153" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="C153" s="5" t="s">
+      <c r="C153" s="3" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A154" s="6"/>
-      <c r="B154" s="5" t="s">
+      <c r="A154" s="11"/>
+      <c r="B154" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="C154" s="5"/>
+      <c r="C154" s="3"/>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A155" s="6"/>
-      <c r="B155" s="5" t="s">
+      <c r="A155" s="11"/>
+      <c r="B155" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="C155" s="5"/>
+      <c r="C155" s="3"/>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B156" s="6"/>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A157">
+      <c r="A157" s="2">
         <v>4</v>
       </c>
-      <c r="B157" s="5" t="s">
+      <c r="B157" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="C157" s="5" t="s">
+      <c r="C157" s="3" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B158" s="5" t="s">
+      <c r="B158" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="C158" s="5" t="s">
+      <c r="C158" s="3" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B159" s="5" t="s">
+      <c r="B159" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="C159" s="5"/>
+      <c r="C159" s="3"/>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B160" s="6"/>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A161" t="s">
+      <c r="A161" s="2" t="s">
         <v>105</v>
       </c>
+      <c r="B161" s="6"/>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A162">
+      <c r="A162" s="2">
         <v>1</v>
       </c>
-      <c r="B162" s="5" t="s">
+      <c r="B162" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="C162" s="5" t="s">
+      <c r="C162" s="3" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B163" s="5" t="s">
+    <row r="163" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B163" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="C163" s="5" t="s">
+      <c r="C163" s="3" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B164" s="5" t="s">
+      <c r="B164" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="C164" s="5" t="s">
+      <c r="C164" s="3" t="s">
         <v>172</v>
       </c>
     </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B165" s="6"/>
+    </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A166">
+      <c r="A166" s="2">
         <v>2</v>
       </c>
-      <c r="B166" s="5" t="s">
+      <c r="B166" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="C166" s="5" t="s">
+      <c r="C166" s="3" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B167" s="5" t="s">
+      <c r="B167" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="C167" s="5" t="s">
+      <c r="C167" s="3" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B168" s="5" t="s">
+      <c r="B168" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="C168" s="5" t="s">
+      <c r="C168" s="3" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B170" s="5"/>
-      <c r="C170" s="5"/>
+      <c r="B170" s="3"/>
+      <c r="C170" s="3"/>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A171" s="6"/>
-      <c r="B171" s="5"/>
-      <c r="C171" s="5"/>
+      <c r="A171" s="11"/>
+      <c r="B171" s="3"/>
+      <c r="C171" s="3"/>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A172" s="6"/>
-      <c r="B172" s="5"/>
-      <c r="C172" s="5"/>
+      <c r="A172" s="11"/>
+      <c r="B172" s="3"/>
+      <c r="C172" s="3"/>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B174" s="5"/>
-      <c r="C174" s="5"/>
+      <c r="B174" s="3"/>
+      <c r="C174" s="3"/>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B175" s="5"/>
-      <c r="C175" s="5"/>
+      <c r="B175" s="3"/>
+      <c r="C175" s="3"/>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B176" s="5"/>
-      <c r="C176" s="5"/>
+      <c r="B176" s="3"/>
+      <c r="C176" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>